<commit_message>
address Prof. Lehmann's comments
</commit_message>
<xml_diff>
--- a/gcam/input/biochar_land_R/GCAM_parameters.xlsx
+++ b/gcam/input/biochar_land_R/GCAM_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\IAM\biochar\gcam\input\biochar_land_R\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{283F6C98-D336-4BFE-ADEB-75140FF7646E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51BBC130-BC02-4A96-BECF-860137C9F5E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{D3FBB104-BEF4-4FDA-A1FA-9751FB33CA85}"/>
+    <workbookView xWindow="510" yWindow="1575" windowWidth="24915" windowHeight="13620" activeTab="1" xr2:uid="{D3FBB104-BEF4-4FDA-A1FA-9751FB33CA85}"/>
   </bookViews>
   <sheets>
     <sheet name="parameter values" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="162">
   <si>
     <t>Name</t>
   </si>
@@ -525,12 +525,6 @@
     <t>BiocharSubsidyHigh</t>
   </si>
   <si>
-    <t>CarbonStabilityLow</t>
-  </si>
-  <si>
-    <t>CarbonStabilityHigh</t>
-  </si>
-  <si>
     <t>Zhou, S., Liang, H., Han, L., Huang, G. and Yang, Z., 2019. The influence of manure feedstock, slow pyrolysis, and hydrothermal temperature on manure thermochemical and combustion properties. Waste management, 88, pp.85-95.</t>
   </si>
   <si>
@@ -562,6 +556,18 @@
   </si>
   <si>
     <t>error</t>
+  </si>
+  <si>
+    <t>to run</t>
+  </si>
+  <si>
+    <t>CarbonPersistenceLow</t>
+  </si>
+  <si>
+    <t>CarbonPersistenceHigh</t>
+  </si>
+  <si>
+    <t>need to update DB, log files, sI figure</t>
   </si>
 </sst>
 </file>
@@ -609,7 +615,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -631,6 +637,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -738,9 +750,9 @@
     <xf numFmtId="9" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1132,13 +1144,13 @@
         <v>65</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="48" thickBot="1" x14ac:dyDescent="0.3">
@@ -1214,13 +1226,13 @@
         <v>65</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="48" thickBot="1" x14ac:dyDescent="0.3">
@@ -1304,7 +1316,7 @@
         <v>6</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1386,7 +1398,7 @@
         <v>6</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="48" thickBot="1" x14ac:dyDescent="0.3">
@@ -1464,7 +1476,7 @@
         <v>6</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="48" thickBot="1" x14ac:dyDescent="0.3">
@@ -1528,13 +1540,13 @@
         <v>21</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>153</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>155</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>34</v>
@@ -1554,13 +1566,13 @@
         <v>22</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>154</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>156</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>34</v>
@@ -2724,7 +2736,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAF4C056-73DD-4AC5-8BE4-76E3645E3B7C}">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
@@ -2732,12 +2744,12 @@
     <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2745,220 +2757,214 @@
         <v>123</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>113</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>102</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>101</v>
       </c>
-      <c r="B5" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>103</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>104</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>111</v>
       </c>
-      <c r="B8" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>112</v>
       </c>
-      <c r="B9" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B9" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>105</v>
       </c>
-      <c r="B10" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B10" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>106</v>
       </c>
-      <c r="B11" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="D11" s="13"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B11" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>107</v>
       </c>
-      <c r="B12" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B12" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>108</v>
       </c>
-      <c r="B13" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>109</v>
       </c>
-      <c r="B14" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B14" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>110</v>
       </c>
-      <c r="B15" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="C15" s="13"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B15" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>124</v>
       </c>
-      <c r="B16" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="C16" s="13"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>125</v>
       </c>
-      <c r="B17" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B17" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>126</v>
       </c>
-      <c r="B18" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="C18" s="13"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B18" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>127</v>
       </c>
-      <c r="B19" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B19" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>114</v>
       </c>
-      <c r="B20" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B20" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>137</v>
       </c>
-      <c r="B21" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B21" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>138</v>
       </c>
-      <c r="B22" s="14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B22" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>143</v>
       </c>
-      <c r="B23" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B23" s="14" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>144</v>
       </c>
-      <c r="B24" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="C24" s="13"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B24" s="14" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>145</v>
       </c>
-      <c r="B25" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="C25" s="13"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B25" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="C25" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>146</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B26" s="14" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>159</v>
       </c>
-      <c r="C26" s="13"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>147</v>
-      </c>
-      <c r="B27" s="14" t="s">
+      <c r="B27" s="15" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>148</v>
-      </c>
-      <c r="B28" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="B28" s="15" t="s">
         <v>158</v>
       </c>
     </row>

</xml_diff>

<commit_message>
new plots and results
</commit_message>
<xml_diff>
--- a/gcam/input/biochar_land_R/GCAM_parameters.xlsx
+++ b/gcam/input/biochar_land_R/GCAM_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\IAM\biochar\gcam\input\biochar_land_R\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51BBC130-BC02-4A96-BECF-860137C9F5E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5664A1A8-22E9-4D95-AD29-60681B7F6033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="510" yWindow="1575" windowWidth="24915" windowHeight="13620" activeTab="1" xr2:uid="{D3FBB104-BEF4-4FDA-A1FA-9751FB33CA85}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="160">
   <si>
     <t>Name</t>
   </si>
@@ -558,16 +558,10 @@
     <t>error</t>
   </si>
   <si>
-    <t>to run</t>
-  </si>
-  <si>
     <t>CarbonPersistenceLow</t>
   </si>
   <si>
     <t>CarbonPersistenceHigh</t>
-  </si>
-  <si>
-    <t>need to update DB, log files, sI figure</t>
   </si>
 </sst>
 </file>
@@ -615,7 +609,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -637,12 +631,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -712,7 +700,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -752,7 +740,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2736,7 +2723,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAF4C056-73DD-4AC5-8BE4-76E3645E3B7C}">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
@@ -2869,7 +2856,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>125</v>
       </c>
@@ -2877,7 +2864,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>126</v>
       </c>
@@ -2885,7 +2872,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>127</v>
       </c>
@@ -2893,7 +2880,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>114</v>
       </c>
@@ -2901,7 +2888,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>137</v>
       </c>
@@ -2909,7 +2896,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>138</v>
       </c>
@@ -2917,7 +2904,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>143</v>
       </c>
@@ -2925,7 +2912,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>144</v>
       </c>
@@ -2933,18 +2920,15 @@
         <v>157</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>145</v>
       </c>
       <c r="B25" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="C25" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>146</v>
       </c>
@@ -2952,20 +2936,20 @@
         <v>157</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>158</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>159</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>160</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>158</v>
+      <c r="B28" s="13" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>